<commit_message>
feat: update export functionality to include operator usernames and submission timestamps in Ahu, CapacitorBank, and EspOperationalReport controllers
</commit_message>
<xml_diff>
--- a/public/assets/templates/operasional/ahu.xlsx
+++ b/public/assets/templates/operasional/ahu.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\laragon\www\pt_bas\Engineering\public\assets\templates\operasional\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C741B628-00DE-44B2-BF5B-327D1EDEBBD7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{10772AB6-B0E1-4D71-B534-03E17EB59812}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10560" xr2:uid="{F42A507E-C648-47AE-8B3F-D3A1A5245282}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="24">
   <si>
     <t>PT BUMI ALAM SEGAR</t>
   </si>
@@ -99,9 +99,6 @@
     <t xml:space="preserve"> SPV Engineering</t>
   </si>
   <si>
-    <t>(                                                            )</t>
-  </si>
-  <si>
     <t>FRM/EUT/01/008/002-04</t>
   </si>
 </sst>
@@ -109,7 +106,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5">
+  <fonts count="7">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -145,6 +142,22 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -596,7 +609,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="75">
+  <cellXfs count="84">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -670,15 +683,56 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="36" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="31" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
@@ -700,19 +754,25 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="35" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="36" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="31" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -745,6 +805,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -788,36 +854,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1183,194 +1219,194 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{512D2555-0C38-4066-8649-1FFA8D5C1D9B}">
-  <dimension ref="A1:AD45"/>
+  <dimension ref="A1:AD46"/>
   <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="14.5"/>
   <sheetData>
     <row r="1" spans="1:30" ht="15" thickTop="1">
-      <c r="A1" s="58"/>
-      <c r="B1" s="59"/>
-      <c r="C1" s="59"/>
-      <c r="D1" s="64" t="s">
+      <c r="A1" s="77"/>
+      <c r="B1" s="78"/>
+      <c r="C1" s="78"/>
+      <c r="D1" s="83" t="s">
         <v>0</v>
       </c>
-      <c r="E1" s="64"/>
-      <c r="F1" s="64"/>
-      <c r="G1" s="64"/>
-      <c r="H1" s="64"/>
-      <c r="I1" s="64"/>
-      <c r="J1" s="64"/>
-      <c r="K1" s="64"/>
-      <c r="L1" s="64"/>
-      <c r="M1" s="64"/>
-      <c r="N1" s="64"/>
-      <c r="O1" s="64"/>
-      <c r="P1" s="64"/>
-      <c r="Q1" s="64"/>
-      <c r="R1" s="64"/>
-      <c r="S1" s="64"/>
-      <c r="T1" s="64"/>
-      <c r="U1" s="65" t="s">
+      <c r="E1" s="83"/>
+      <c r="F1" s="83"/>
+      <c r="G1" s="83"/>
+      <c r="H1" s="83"/>
+      <c r="I1" s="83"/>
+      <c r="J1" s="83"/>
+      <c r="K1" s="83"/>
+      <c r="L1" s="83"/>
+      <c r="M1" s="83"/>
+      <c r="N1" s="83"/>
+      <c r="O1" s="83"/>
+      <c r="P1" s="83"/>
+      <c r="Q1" s="83"/>
+      <c r="R1" s="83"/>
+      <c r="S1" s="83"/>
+      <c r="T1" s="83"/>
+      <c r="U1" s="39" t="s">
         <v>1</v>
       </c>
-      <c r="V1" s="66"/>
-      <c r="W1" s="69"/>
-      <c r="X1" s="70"/>
-      <c r="Y1" s="70"/>
-      <c r="Z1" s="70"/>
-      <c r="AA1" s="70"/>
-      <c r="AB1" s="70"/>
-      <c r="AC1" s="70"/>
-      <c r="AD1" s="71"/>
+      <c r="V1" s="40"/>
+      <c r="W1" s="51"/>
+      <c r="X1" s="52"/>
+      <c r="Y1" s="52"/>
+      <c r="Z1" s="52"/>
+      <c r="AA1" s="52"/>
+      <c r="AB1" s="52"/>
+      <c r="AC1" s="52"/>
+      <c r="AD1" s="53"/>
     </row>
     <row r="2" spans="1:30">
-      <c r="A2" s="60"/>
-      <c r="B2" s="61"/>
-      <c r="C2" s="61"/>
-      <c r="D2" s="40"/>
-      <c r="E2" s="40"/>
-      <c r="F2" s="40"/>
-      <c r="G2" s="40"/>
-      <c r="H2" s="40"/>
-      <c r="I2" s="40"/>
-      <c r="J2" s="40"/>
-      <c r="K2" s="40"/>
-      <c r="L2" s="40"/>
-      <c r="M2" s="40"/>
-      <c r="N2" s="40"/>
-      <c r="O2" s="40"/>
-      <c r="P2" s="40"/>
-      <c r="Q2" s="40"/>
-      <c r="R2" s="40"/>
-      <c r="S2" s="40"/>
-      <c r="T2" s="40"/>
-      <c r="U2" s="67"/>
-      <c r="V2" s="68"/>
-      <c r="W2" s="72"/>
-      <c r="X2" s="73"/>
-      <c r="Y2" s="73"/>
-      <c r="Z2" s="73"/>
-      <c r="AA2" s="73"/>
-      <c r="AB2" s="73"/>
-      <c r="AC2" s="73"/>
-      <c r="AD2" s="74"/>
+      <c r="A2" s="79"/>
+      <c r="B2" s="80"/>
+      <c r="C2" s="80"/>
+      <c r="D2" s="57"/>
+      <c r="E2" s="57"/>
+      <c r="F2" s="57"/>
+      <c r="G2" s="57"/>
+      <c r="H2" s="57"/>
+      <c r="I2" s="57"/>
+      <c r="J2" s="57"/>
+      <c r="K2" s="57"/>
+      <c r="L2" s="57"/>
+      <c r="M2" s="57"/>
+      <c r="N2" s="57"/>
+      <c r="O2" s="57"/>
+      <c r="P2" s="57"/>
+      <c r="Q2" s="57"/>
+      <c r="R2" s="57"/>
+      <c r="S2" s="57"/>
+      <c r="T2" s="57"/>
+      <c r="U2" s="41"/>
+      <c r="V2" s="42"/>
+      <c r="W2" s="54"/>
+      <c r="X2" s="55"/>
+      <c r="Y2" s="55"/>
+      <c r="Z2" s="55"/>
+      <c r="AA2" s="55"/>
+      <c r="AB2" s="55"/>
+      <c r="AC2" s="55"/>
+      <c r="AD2" s="56"/>
     </row>
     <row r="3" spans="1:30">
-      <c r="A3" s="60"/>
-      <c r="B3" s="61"/>
-      <c r="C3" s="61"/>
-      <c r="D3" s="40" t="s">
+      <c r="A3" s="79"/>
+      <c r="B3" s="80"/>
+      <c r="C3" s="80"/>
+      <c r="D3" s="57" t="s">
         <v>2</v>
       </c>
-      <c r="E3" s="40"/>
-      <c r="F3" s="40"/>
-      <c r="G3" s="40"/>
-      <c r="H3" s="40"/>
-      <c r="I3" s="40"/>
-      <c r="J3" s="40"/>
-      <c r="K3" s="40"/>
-      <c r="L3" s="40"/>
-      <c r="M3" s="40"/>
-      <c r="N3" s="40"/>
-      <c r="O3" s="40"/>
-      <c r="P3" s="40"/>
-      <c r="Q3" s="40"/>
-      <c r="R3" s="40"/>
-      <c r="S3" s="40"/>
-      <c r="T3" s="40"/>
-      <c r="U3" s="42" t="s">
+      <c r="E3" s="57"/>
+      <c r="F3" s="57"/>
+      <c r="G3" s="57"/>
+      <c r="H3" s="57"/>
+      <c r="I3" s="57"/>
+      <c r="J3" s="57"/>
+      <c r="K3" s="57"/>
+      <c r="L3" s="57"/>
+      <c r="M3" s="57"/>
+      <c r="N3" s="57"/>
+      <c r="O3" s="57"/>
+      <c r="P3" s="57"/>
+      <c r="Q3" s="57"/>
+      <c r="R3" s="57"/>
+      <c r="S3" s="57"/>
+      <c r="T3" s="57"/>
+      <c r="U3" s="59" t="s">
         <v>3</v>
       </c>
-      <c r="V3" s="43"/>
-      <c r="W3" s="46"/>
-      <c r="X3" s="47"/>
-      <c r="Y3" s="47"/>
-      <c r="Z3" s="47"/>
-      <c r="AA3" s="47"/>
-      <c r="AB3" s="47"/>
-      <c r="AC3" s="47"/>
-      <c r="AD3" s="48"/>
+      <c r="V3" s="60"/>
+      <c r="W3" s="63"/>
+      <c r="X3" s="64"/>
+      <c r="Y3" s="64"/>
+      <c r="Z3" s="64"/>
+      <c r="AA3" s="64"/>
+      <c r="AB3" s="64"/>
+      <c r="AC3" s="64"/>
+      <c r="AD3" s="65"/>
     </row>
     <row r="4" spans="1:30" ht="40" customHeight="1" thickBot="1">
-      <c r="A4" s="62"/>
-      <c r="B4" s="63"/>
-      <c r="C4" s="63"/>
-      <c r="D4" s="41"/>
-      <c r="E4" s="41"/>
-      <c r="F4" s="41"/>
-      <c r="G4" s="41"/>
-      <c r="H4" s="41"/>
-      <c r="I4" s="41"/>
-      <c r="J4" s="41"/>
-      <c r="K4" s="41"/>
-      <c r="L4" s="41"/>
-      <c r="M4" s="41"/>
-      <c r="N4" s="41"/>
-      <c r="O4" s="41"/>
-      <c r="P4" s="41"/>
-      <c r="Q4" s="41"/>
-      <c r="R4" s="41"/>
-      <c r="S4" s="41"/>
-      <c r="T4" s="41"/>
-      <c r="U4" s="44"/>
-      <c r="V4" s="45"/>
-      <c r="W4" s="49"/>
-      <c r="X4" s="38"/>
-      <c r="Y4" s="38"/>
-      <c r="Z4" s="38"/>
-      <c r="AA4" s="38"/>
-      <c r="AB4" s="38"/>
-      <c r="AC4" s="38"/>
-      <c r="AD4" s="39"/>
+      <c r="A4" s="81"/>
+      <c r="B4" s="82"/>
+      <c r="C4" s="82"/>
+      <c r="D4" s="58"/>
+      <c r="E4" s="58"/>
+      <c r="F4" s="58"/>
+      <c r="G4" s="58"/>
+      <c r="H4" s="58"/>
+      <c r="I4" s="58"/>
+      <c r="J4" s="58"/>
+      <c r="K4" s="58"/>
+      <c r="L4" s="58"/>
+      <c r="M4" s="58"/>
+      <c r="N4" s="58"/>
+      <c r="O4" s="58"/>
+      <c r="P4" s="58"/>
+      <c r="Q4" s="58"/>
+      <c r="R4" s="58"/>
+      <c r="S4" s="58"/>
+      <c r="T4" s="58"/>
+      <c r="U4" s="61"/>
+      <c r="V4" s="62"/>
+      <c r="W4" s="66"/>
+      <c r="X4" s="67"/>
+      <c r="Y4" s="67"/>
+      <c r="Z4" s="67"/>
+      <c r="AA4" s="67"/>
+      <c r="AB4" s="67"/>
+      <c r="AC4" s="67"/>
+      <c r="AD4" s="68"/>
     </row>
     <row r="5" spans="1:30" ht="15" thickTop="1">
-      <c r="A5" s="50" t="s">
+      <c r="A5" s="69" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="52" t="s">
+      <c r="B5" s="71" t="s">
         <v>5</v>
       </c>
-      <c r="C5" s="54" t="s">
+      <c r="C5" s="73" t="s">
         <v>6</v>
       </c>
-      <c r="D5" s="55"/>
-      <c r="E5" s="55"/>
-      <c r="F5" s="55"/>
-      <c r="G5" s="55"/>
-      <c r="H5" s="56"/>
-      <c r="I5" s="54" t="s">
+      <c r="D5" s="74"/>
+      <c r="E5" s="74"/>
+      <c r="F5" s="74"/>
+      <c r="G5" s="74"/>
+      <c r="H5" s="75"/>
+      <c r="I5" s="73" t="s">
         <v>7</v>
       </c>
-      <c r="J5" s="55"/>
-      <c r="K5" s="55"/>
-      <c r="L5" s="55"/>
-      <c r="M5" s="55"/>
-      <c r="N5" s="56"/>
-      <c r="O5" s="54" t="s">
+      <c r="J5" s="74"/>
+      <c r="K5" s="74"/>
+      <c r="L5" s="74"/>
+      <c r="M5" s="74"/>
+      <c r="N5" s="75"/>
+      <c r="O5" s="73" t="s">
         <v>8</v>
       </c>
-      <c r="P5" s="55"/>
-      <c r="Q5" s="55"/>
-      <c r="R5" s="55"/>
-      <c r="S5" s="55"/>
-      <c r="T5" s="56"/>
-      <c r="U5" s="54" t="s">
+      <c r="P5" s="74"/>
+      <c r="Q5" s="74"/>
+      <c r="R5" s="74"/>
+      <c r="S5" s="74"/>
+      <c r="T5" s="75"/>
+      <c r="U5" s="73" t="s">
         <v>9</v>
       </c>
-      <c r="V5" s="55"/>
-      <c r="W5" s="55"/>
-      <c r="X5" s="55"/>
-      <c r="Y5" s="55"/>
-      <c r="Z5" s="56"/>
-      <c r="AA5" s="55" t="s">
+      <c r="V5" s="74"/>
+      <c r="W5" s="74"/>
+      <c r="X5" s="74"/>
+      <c r="Y5" s="74"/>
+      <c r="Z5" s="75"/>
+      <c r="AA5" s="74" t="s">
         <v>10</v>
       </c>
-      <c r="AB5" s="55"/>
-      <c r="AC5" s="55"/>
-      <c r="AD5" s="57"/>
+      <c r="AB5" s="74"/>
+      <c r="AC5" s="74"/>
+      <c r="AD5" s="76"/>
     </row>
     <row r="6" spans="1:30" ht="21">
-      <c r="A6" s="51"/>
-      <c r="B6" s="53"/>
+      <c r="A6" s="70"/>
+      <c r="B6" s="72"/>
       <c r="C6" s="8" t="s">
         <v>11</v>
       </c>
@@ -2511,84 +2547,84 @@
       <c r="AD37" s="19"/>
     </row>
     <row r="38" spans="1:30" ht="15.5" thickTop="1" thickBot="1">
-      <c r="A38" s="28" t="s">
+      <c r="A38" s="43" t="s">
         <v>18</v>
       </c>
-      <c r="B38" s="29"/>
-      <c r="C38" s="29"/>
+      <c r="B38" s="44"/>
+      <c r="C38" s="44"/>
       <c r="D38" s="20"/>
-      <c r="E38" s="30" t="s">
+      <c r="E38" s="45" t="s">
         <v>19</v>
       </c>
-      <c r="F38" s="31"/>
-      <c r="G38" s="31"/>
-      <c r="H38" s="31"/>
-      <c r="I38" s="31"/>
-      <c r="J38" s="31"/>
-      <c r="K38" s="31"/>
-      <c r="L38" s="31"/>
-      <c r="M38" s="31"/>
-      <c r="N38" s="31"/>
-      <c r="O38" s="31"/>
-      <c r="P38" s="31"/>
-      <c r="Q38" s="31"/>
-      <c r="R38" s="31"/>
-      <c r="S38" s="31"/>
-      <c r="T38" s="31"/>
-      <c r="U38" s="31"/>
-      <c r="V38" s="31"/>
-      <c r="W38" s="31"/>
-      <c r="X38" s="31"/>
-      <c r="Y38" s="31"/>
-      <c r="Z38" s="31"/>
-      <c r="AA38" s="31"/>
-      <c r="AB38" s="31"/>
-      <c r="AC38" s="32"/>
-      <c r="AD38" s="33"/>
+      <c r="F38" s="46"/>
+      <c r="G38" s="46"/>
+      <c r="H38" s="46"/>
+      <c r="I38" s="46"/>
+      <c r="J38" s="46"/>
+      <c r="K38" s="46"/>
+      <c r="L38" s="46"/>
+      <c r="M38" s="46"/>
+      <c r="N38" s="46"/>
+      <c r="O38" s="46"/>
+      <c r="P38" s="46"/>
+      <c r="Q38" s="46"/>
+      <c r="R38" s="46"/>
+      <c r="S38" s="46"/>
+      <c r="T38" s="46"/>
+      <c r="U38" s="46"/>
+      <c r="V38" s="46"/>
+      <c r="W38" s="46"/>
+      <c r="X38" s="46"/>
+      <c r="Y38" s="46"/>
+      <c r="Z38" s="46"/>
+      <c r="AA38" s="46"/>
+      <c r="AB38" s="46"/>
+      <c r="AC38" s="47"/>
+      <c r="AD38" s="48"/>
     </row>
     <row r="39" spans="1:30" ht="15" thickTop="1">
-      <c r="A39" s="34" t="s">
+      <c r="A39" s="49" t="s">
         <v>20</v>
       </c>
-      <c r="B39" s="35"/>
-      <c r="C39" s="35"/>
-      <c r="D39" s="35"/>
-      <c r="E39" s="35"/>
+      <c r="B39" s="37"/>
+      <c r="C39" s="37"/>
+      <c r="D39" s="37"/>
+      <c r="E39" s="37"/>
       <c r="F39" s="23"/>
       <c r="G39" s="23"/>
       <c r="H39" s="23"/>
       <c r="I39" s="23"/>
       <c r="J39" s="23"/>
-      <c r="K39" s="35" t="s">
+      <c r="K39" s="37" t="s">
         <v>21</v>
       </c>
-      <c r="L39" s="35"/>
-      <c r="M39" s="35"/>
-      <c r="N39" s="35"/>
-      <c r="O39" s="35"/>
-      <c r="P39" s="35"/>
-      <c r="Q39" s="35"/>
+      <c r="L39" s="37"/>
+      <c r="M39" s="37"/>
+      <c r="N39" s="37"/>
+      <c r="O39" s="37"/>
+      <c r="P39" s="37"/>
+      <c r="Q39" s="37"/>
       <c r="R39" s="23"/>
       <c r="S39" s="23"/>
       <c r="T39" s="23"/>
       <c r="U39" s="23"/>
       <c r="V39" s="23"/>
       <c r="W39" s="23"/>
-      <c r="X39" s="35" t="s">
+      <c r="X39" s="37" t="s">
         <v>22</v>
       </c>
-      <c r="Y39" s="35"/>
-      <c r="Z39" s="35"/>
-      <c r="AA39" s="35"/>
-      <c r="AB39" s="35"/>
-      <c r="AC39" s="35"/>
-      <c r="AD39" s="36"/>
+      <c r="Y39" s="37"/>
+      <c r="Z39" s="37"/>
+      <c r="AA39" s="37"/>
+      <c r="AB39" s="37"/>
+      <c r="AC39" s="37"/>
+      <c r="AD39" s="50"/>
     </row>
     <row r="40" spans="1:30">
       <c r="A40" s="21"/>
-      <c r="B40" s="22"/>
-      <c r="C40" s="23"/>
-      <c r="D40" s="23"/>
+      <c r="B40" s="37"/>
+      <c r="C40" s="37"/>
+      <c r="D40" s="37"/>
       <c r="E40" s="23"/>
       <c r="F40" s="23"/>
       <c r="G40" s="23"/>
@@ -2597,9 +2633,9 @@
       <c r="J40" s="23"/>
       <c r="K40" s="23"/>
       <c r="L40" s="22"/>
-      <c r="M40" s="23"/>
-      <c r="N40" s="23"/>
-      <c r="O40" s="23"/>
+      <c r="M40" s="37"/>
+      <c r="N40" s="37"/>
+      <c r="O40" s="37"/>
       <c r="P40" s="23"/>
       <c r="Q40" s="22"/>
       <c r="R40" s="22"/>
@@ -2610,17 +2646,17 @@
       <c r="W40" s="23"/>
       <c r="X40" s="23"/>
       <c r="Y40" s="23"/>
-      <c r="Z40" s="23"/>
-      <c r="AA40" s="23"/>
-      <c r="AB40" s="23"/>
+      <c r="Z40" s="37"/>
+      <c r="AA40" s="37"/>
+      <c r="AB40" s="37"/>
       <c r="AC40" s="23"/>
       <c r="AD40" s="24"/>
     </row>
     <row r="41" spans="1:30">
       <c r="A41" s="21"/>
-      <c r="B41" s="22"/>
-      <c r="C41" s="23"/>
-      <c r="D41" s="23"/>
+      <c r="B41" s="37"/>
+      <c r="C41" s="37"/>
+      <c r="D41" s="37"/>
       <c r="E41" s="23"/>
       <c r="F41" s="23"/>
       <c r="G41" s="23"/>
@@ -2629,9 +2665,9 @@
       <c r="J41" s="23"/>
       <c r="K41" s="23"/>
       <c r="L41" s="22"/>
-      <c r="M41" s="23"/>
-      <c r="N41" s="23"/>
-      <c r="O41" s="23"/>
+      <c r="M41" s="37"/>
+      <c r="N41" s="37"/>
+      <c r="O41" s="37"/>
       <c r="P41" s="23"/>
       <c r="Q41" s="22"/>
       <c r="R41" s="22"/>
@@ -2642,17 +2678,17 @@
       <c r="W41" s="23"/>
       <c r="X41" s="23"/>
       <c r="Y41" s="23"/>
-      <c r="Z41" s="23"/>
-      <c r="AA41" s="23"/>
-      <c r="AB41" s="23"/>
+      <c r="Z41" s="37"/>
+      <c r="AA41" s="37"/>
+      <c r="AB41" s="37"/>
       <c r="AC41" s="23"/>
       <c r="AD41" s="24"/>
     </row>
     <row r="42" spans="1:30">
       <c r="A42" s="21"/>
-      <c r="B42" s="22"/>
-      <c r="C42" s="23"/>
-      <c r="D42" s="23"/>
+      <c r="B42" s="37"/>
+      <c r="C42" s="37"/>
+      <c r="D42" s="37"/>
       <c r="E42" s="23"/>
       <c r="F42" s="23"/>
       <c r="G42" s="23"/>
@@ -2661,9 +2697,9 @@
       <c r="J42" s="23"/>
       <c r="K42" s="23"/>
       <c r="L42" s="22"/>
-      <c r="M42" s="23"/>
-      <c r="N42" s="23"/>
-      <c r="O42" s="23"/>
+      <c r="M42" s="37"/>
+      <c r="N42" s="37"/>
+      <c r="O42" s="37"/>
       <c r="P42" s="23"/>
       <c r="Q42" s="22"/>
       <c r="R42" s="22"/>
@@ -2674,17 +2710,17 @@
       <c r="W42" s="23"/>
       <c r="X42" s="23"/>
       <c r="Y42" s="23"/>
-      <c r="Z42" s="23"/>
-      <c r="AA42" s="23"/>
-      <c r="AB42" s="23"/>
+      <c r="Z42" s="37"/>
+      <c r="AA42" s="37"/>
+      <c r="AB42" s="37"/>
       <c r="AC42" s="23"/>
       <c r="AD42" s="24"/>
     </row>
     <row r="43" spans="1:30">
       <c r="A43" s="21"/>
-      <c r="B43" s="22"/>
-      <c r="C43" s="23"/>
-      <c r="D43" s="23"/>
+      <c r="B43" s="37"/>
+      <c r="C43" s="37"/>
+      <c r="D43" s="37"/>
       <c r="E43" s="23"/>
       <c r="F43" s="23"/>
       <c r="G43" s="23"/>
@@ -2693,9 +2729,9 @@
       <c r="J43" s="23"/>
       <c r="K43" s="23"/>
       <c r="L43" s="22"/>
-      <c r="M43" s="23"/>
-      <c r="N43" s="23"/>
-      <c r="O43" s="23"/>
+      <c r="M43" s="37"/>
+      <c r="N43" s="37"/>
+      <c r="O43" s="37"/>
       <c r="P43" s="23"/>
       <c r="Q43" s="22"/>
       <c r="R43" s="22"/>
@@ -2706,90 +2742,122 @@
       <c r="W43" s="23"/>
       <c r="X43" s="23"/>
       <c r="Y43" s="23"/>
-      <c r="Z43" s="23"/>
-      <c r="AA43" s="23"/>
-      <c r="AB43" s="23"/>
+      <c r="Z43" s="37"/>
+      <c r="AA43" s="37"/>
+      <c r="AB43" s="37"/>
       <c r="AC43" s="23"/>
       <c r="AD43" s="24"/>
     </row>
-    <row r="44" spans="1:30" ht="15" thickBot="1">
-      <c r="A44" s="37" t="s">
-        <v>23</v>
-      </c>
+    <row r="44" spans="1:30" s="35" customFormat="1">
+      <c r="A44" s="31"/>
       <c r="B44" s="38"/>
       <c r="C44" s="38"/>
       <c r="D44" s="38"/>
-      <c r="E44" s="38"/>
-      <c r="F44" s="25"/>
-      <c r="G44" s="25"/>
-      <c r="H44" s="25"/>
-      <c r="I44" s="25"/>
-      <c r="J44" s="25"/>
-      <c r="K44" s="38" t="s">
-        <v>23</v>
-      </c>
-      <c r="L44" s="38"/>
+      <c r="E44" s="33"/>
+      <c r="F44" s="33"/>
+      <c r="G44" s="33"/>
+      <c r="H44" s="32"/>
+      <c r="I44" s="33"/>
+      <c r="J44" s="33"/>
+      <c r="K44" s="33"/>
+      <c r="L44" s="32"/>
       <c r="M44" s="38"/>
       <c r="N44" s="38"/>
       <c r="O44" s="38"/>
-      <c r="P44" s="38"/>
-      <c r="Q44" s="38"/>
-      <c r="R44" s="25"/>
-      <c r="S44" s="25"/>
-      <c r="T44" s="25"/>
-      <c r="U44" s="25"/>
-      <c r="V44" s="25"/>
-      <c r="W44" s="25"/>
-      <c r="X44" s="38" t="s">
-        <v>23</v>
-      </c>
-      <c r="Y44" s="38"/>
+      <c r="P44" s="33"/>
+      <c r="Q44" s="32"/>
+      <c r="R44" s="32"/>
+      <c r="S44" s="33"/>
+      <c r="T44" s="33"/>
+      <c r="U44" s="33"/>
+      <c r="V44" s="33"/>
+      <c r="W44" s="33"/>
+      <c r="X44" s="33"/>
+      <c r="Y44" s="33"/>
       <c r="Z44" s="38"/>
       <c r="AA44" s="38"/>
       <c r="AB44" s="38"/>
-      <c r="AC44" s="38"/>
-      <c r="AD44" s="39"/>
-    </row>
-    <row r="45" spans="1:30" ht="15" thickTop="1">
-      <c r="A45" s="22"/>
-      <c r="B45" s="23"/>
-      <c r="C45" s="23"/>
-      <c r="D45" s="23"/>
-      <c r="E45" s="23"/>
-      <c r="F45" s="23"/>
-      <c r="G45" s="23"/>
-      <c r="H45" s="23"/>
-      <c r="I45" s="23"/>
-      <c r="J45" s="23"/>
-      <c r="K45" s="23"/>
-      <c r="L45" s="23"/>
-      <c r="M45" s="23"/>
-      <c r="N45" s="23"/>
-      <c r="O45" s="23"/>
-      <c r="P45" s="23"/>
-      <c r="Q45" s="23"/>
-      <c r="R45" s="23"/>
-      <c r="S45" s="23"/>
-      <c r="T45" s="23"/>
-      <c r="U45" s="23"/>
-      <c r="V45" s="23"/>
-      <c r="W45" s="23"/>
-      <c r="X45" s="26"/>
-      <c r="Y45" s="23"/>
-      <c r="Z45" s="26"/>
-      <c r="AA45" s="26" t="s">
-        <v>24</v>
-      </c>
-      <c r="AB45" s="26"/>
-      <c r="AC45" s="26"/>
-      <c r="AD45" s="27"/>
+      <c r="AC44" s="33"/>
+      <c r="AD44" s="34"/>
+    </row>
+    <row r="45" spans="1:30" s="30" customFormat="1" ht="15" thickBot="1">
+      <c r="A45" s="27"/>
+      <c r="B45" s="36"/>
+      <c r="C45" s="36"/>
+      <c r="D45" s="36"/>
+      <c r="E45" s="28"/>
+      <c r="F45" s="28"/>
+      <c r="G45" s="28"/>
+      <c r="H45" s="28"/>
+      <c r="I45" s="28"/>
+      <c r="J45" s="28"/>
+      <c r="K45" s="28"/>
+      <c r="L45" s="28"/>
+      <c r="M45" s="36"/>
+      <c r="N45" s="36"/>
+      <c r="O45" s="36"/>
+      <c r="P45" s="28"/>
+      <c r="Q45" s="28"/>
+      <c r="R45" s="28"/>
+      <c r="S45" s="28"/>
+      <c r="T45" s="28"/>
+      <c r="U45" s="28"/>
+      <c r="V45" s="28"/>
+      <c r="W45" s="28"/>
+      <c r="X45" s="28"/>
+      <c r="Y45" s="28"/>
+      <c r="Z45" s="36"/>
+      <c r="AA45" s="36"/>
+      <c r="AB45" s="36"/>
+      <c r="AC45" s="28"/>
+      <c r="AD45" s="29"/>
+    </row>
+    <row r="46" spans="1:30" ht="15" thickTop="1">
+      <c r="A46" s="22"/>
+      <c r="B46" s="23"/>
+      <c r="C46" s="23"/>
+      <c r="D46" s="23"/>
+      <c r="E46" s="23"/>
+      <c r="F46" s="23"/>
+      <c r="G46" s="23"/>
+      <c r="H46" s="23"/>
+      <c r="I46" s="23"/>
+      <c r="J46" s="23"/>
+      <c r="K46" s="23"/>
+      <c r="L46" s="23"/>
+      <c r="M46" s="23"/>
+      <c r="N46" s="23"/>
+      <c r="O46" s="23"/>
+      <c r="P46" s="23"/>
+      <c r="Q46" s="23"/>
+      <c r="R46" s="23"/>
+      <c r="S46" s="23"/>
+      <c r="T46" s="23"/>
+      <c r="U46" s="23"/>
+      <c r="V46" s="23"/>
+      <c r="W46" s="23"/>
+      <c r="X46" s="25"/>
+      <c r="Y46" s="23"/>
+      <c r="Z46" s="25"/>
+      <c r="AA46" s="25" t="s">
+        <v>23</v>
+      </c>
+      <c r="AB46" s="25"/>
+      <c r="AC46" s="25"/>
+      <c r="AD46" s="26"/>
     </row>
   </sheetData>
-  <mergeCells count="22">
+  <mergeCells count="28">
+    <mergeCell ref="AA5:AD5"/>
+    <mergeCell ref="A1:C4"/>
+    <mergeCell ref="D1:T2"/>
+    <mergeCell ref="U1:V2"/>
+    <mergeCell ref="A38:C38"/>
+    <mergeCell ref="E38:AD38"/>
+    <mergeCell ref="A39:E39"/>
+    <mergeCell ref="K39:Q39"/>
+    <mergeCell ref="X39:AD39"/>
     <mergeCell ref="W1:AD2"/>
-    <mergeCell ref="A44:E44"/>
-    <mergeCell ref="K44:Q44"/>
-    <mergeCell ref="X44:AD44"/>
     <mergeCell ref="D3:T4"/>
     <mergeCell ref="U3:V4"/>
     <mergeCell ref="W3:AD4"/>
@@ -2799,15 +2867,15 @@
     <mergeCell ref="I5:N5"/>
     <mergeCell ref="O5:T5"/>
     <mergeCell ref="U5:Z5"/>
-    <mergeCell ref="AA5:AD5"/>
-    <mergeCell ref="A1:C4"/>
-    <mergeCell ref="D1:T2"/>
-    <mergeCell ref="U1:V2"/>
-    <mergeCell ref="A38:C38"/>
-    <mergeCell ref="E38:AD38"/>
-    <mergeCell ref="A39:E39"/>
-    <mergeCell ref="K39:Q39"/>
-    <mergeCell ref="X39:AD39"/>
+    <mergeCell ref="B45:D45"/>
+    <mergeCell ref="M45:O45"/>
+    <mergeCell ref="Z45:AB45"/>
+    <mergeCell ref="B40:D43"/>
+    <mergeCell ref="B44:D44"/>
+    <mergeCell ref="M40:O43"/>
+    <mergeCell ref="M44:O44"/>
+    <mergeCell ref="Z40:AB43"/>
+    <mergeCell ref="Z44:AB44"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing r:id="rId1"/>

</xml_diff>